<commit_message>
fix(forward): purificar grade de 06/10 com apenas jogos certos e liquidar 05/10
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-05.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-05.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -664,15 +664,19 @@
       <c r="K3" t="n">
         <v>1.47</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">

</xml_diff>